<commit_message>
Update Excel sheets with normalized priority and latest sync data
</commit_message>
<xml_diff>
--- a/Inventory Detail (1).xlsx
+++ b/Inventory Detail (1).xlsx
@@ -38049,7 +38049,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A944DE7E-347B-4FB3-BB48-83C558A35775}</x14:id>
+          <x14:id>{E2617EF5-3590-4F7F-8CAC-51465D0E8AAD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38063,7 +38063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49FB744E-CCA2-4DA3-998E-05CD45FE64B8}</x14:id>
+          <x14:id>{E9F8CD34-D047-4900-B8A9-B68EC470A106}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38077,7 +38077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8BB1587D-AB35-4CC2-99D4-A238695BA4A2}</x14:id>
+          <x14:id>{8160DC6C-45AD-447E-89D9-52704ABBA3E4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38091,7 +38091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1C609605-45CA-4050-B18E-03384411C58B}</x14:id>
+          <x14:id>{59EDB521-FF35-4F5B-9F20-2C1DAC5F964F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38105,7 +38105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2DA3CD02-9CAB-44D2-B4A7-40EE4406D362}</x14:id>
+          <x14:id>{FBCD0D26-2697-4443-BBED-A76709ED31F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38119,7 +38119,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8A22510D-3A89-4042-9103-BBEA07A36E58}</x14:id>
+          <x14:id>{09536EE1-EDA5-4A51-9566-92934FFF9FD2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38133,7 +38133,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{907E40D2-6CB9-4439-98F8-4689D1B97FC6}</x14:id>
+          <x14:id>{1253CBFB-27AF-4632-B3D8-B81CAFFED00F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38147,7 +38147,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A5670326-9C97-4E17-B8C1-D59074D22C6C}</x14:id>
+          <x14:id>{B3E0D2E2-133A-4A13-AF04-B45E9BCBD6DE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38161,7 +38161,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B0F0D91A-7B28-4AE1-A798-0967889A27A0}</x14:id>
+          <x14:id>{319BF263-6BDD-456C-BD94-188FCD6E804A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38175,7 +38175,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C35499B0-87F8-4A11-A8B7-ABCE41C6B181}</x14:id>
+          <x14:id>{E6E8DD67-3771-4B4A-A563-43B111B89B91}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38189,7 +38189,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{657E11A8-B579-431F-8102-036525F5C3AA}</x14:id>
+          <x14:id>{6DC4E869-056E-4E88-9747-FEA43BDFC0AD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38203,7 +38203,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CDF86CAB-2690-41B6-AAB3-96A4E0EC946F}</x14:id>
+          <x14:id>{A8A4D78D-261C-4D26-8AFF-CDC1169781FF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38217,7 +38217,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FC56720C-3B19-46AE-8838-DDE8784FF802}</x14:id>
+          <x14:id>{B16B48F3-484B-41E3-8248-0D09A99D63A7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -38228,7 +38228,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A944DE7E-347B-4FB3-BB48-83C558A35775}">
+          <x14:cfRule type="dataBar" id="{E2617EF5-3590-4F7F-8CAC-51465D0E8AAD}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38239,7 +38239,7 @@
           <xm:sqref>E209</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49FB744E-CCA2-4DA3-998E-05CD45FE64B8}">
+          <x14:cfRule type="dataBar" id="{E9F8CD34-D047-4900-B8A9-B68EC470A106}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38250,7 +38250,7 @@
           <xm:sqref>E210</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8BB1587D-AB35-4CC2-99D4-A238695BA4A2}">
+          <x14:cfRule type="dataBar" id="{8160DC6C-45AD-447E-89D9-52704ABBA3E4}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38261,7 +38261,7 @@
           <xm:sqref>E233</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1C609605-45CA-4050-B18E-03384411C58B}">
+          <x14:cfRule type="dataBar" id="{59EDB521-FF35-4F5B-9F20-2C1DAC5F964F}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38272,7 +38272,7 @@
           <xm:sqref>E234</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2DA3CD02-9CAB-44D2-B4A7-40EE4406D362}">
+          <x14:cfRule type="dataBar" id="{FBCD0D26-2697-4443-BBED-A76709ED31F5}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38283,7 +38283,7 @@
           <xm:sqref>E302</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8A22510D-3A89-4042-9103-BBEA07A36E58}">
+          <x14:cfRule type="dataBar" id="{09536EE1-EDA5-4A51-9566-92934FFF9FD2}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38294,7 +38294,7 @@
           <xm:sqref>E303</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{907E40D2-6CB9-4439-98F8-4689D1B97FC6}">
+          <x14:cfRule type="dataBar" id="{1253CBFB-27AF-4632-B3D8-B81CAFFED00F}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38305,7 +38305,7 @@
           <xm:sqref>E575</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A5670326-9C97-4E17-B8C1-D59074D22C6C}">
+          <x14:cfRule type="dataBar" id="{B3E0D2E2-133A-4A13-AF04-B45E9BCBD6DE}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38316,7 +38316,7 @@
           <xm:sqref>E576</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B0F0D91A-7B28-4AE1-A798-0967889A27A0}">
+          <x14:cfRule type="dataBar" id="{319BF263-6BDD-456C-BD94-188FCD6E804A}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38327,7 +38327,7 @@
           <xm:sqref>E1017</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C35499B0-87F8-4A11-A8B7-ABCE41C6B181}">
+          <x14:cfRule type="dataBar" id="{E6E8DD67-3771-4B4A-A563-43B111B89B91}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38338,7 +38338,7 @@
           <xm:sqref>E1018</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{657E11A8-B579-431F-8102-036525F5C3AA}">
+          <x14:cfRule type="dataBar" id="{6DC4E869-056E-4E88-9747-FEA43BDFC0AD}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38349,7 +38349,7 @@
           <xm:sqref>E1065</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CDF86CAB-2690-41B6-AAB3-96A4E0EC946F}">
+          <x14:cfRule type="dataBar" id="{A8A4D78D-261C-4D26-8AFF-CDC1169781FF}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -38360,7 +38360,7 @@
           <xm:sqref>E1066</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FC56720C-3B19-46AE-8838-DDE8784FF802}">
+          <x14:cfRule type="dataBar" id="{B16B48F3-484B-41E3-8248-0D09A99D63A7}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>